<commit_message>
feat(school-students): auto-set school_origin from school profile and reject invalid import with 422
</commit_message>
<xml_diff>
--- a/requests/sample-files/data-siswa.xlsx
+++ b/requests/sample-files/data-siswa.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>full_name</t>
   </si>
@@ -26,97 +26,43 @@
     <t>major</t>
   </si>
   <si>
-    <t>school_origin</t>
-  </si>
-  <si>
     <t>graduation_status</t>
   </si>
   <si>
     <t>class_year</t>
   </si>
   <si>
-    <t>phone_number</t>
-  </si>
-  <si>
     <t>address</t>
   </si>
   <si>
-    <t>Dewi Lestari</t>
-  </si>
-  <si>
-    <t>2000000001</t>
+    <t>Rina Amelia</t>
+  </si>
+  <si>
+    <t>Teknik Komputer dan Jaringan</t>
+  </si>
+  <si>
+    <t>Belum Lulus</t>
+  </si>
+  <si>
+    <t>Jl. Contoh No. 1, Jakarta</t>
+  </si>
+  <si>
+    <t>Dimas Prasetyo</t>
   </si>
   <si>
     <t>Rekayasa Perangkat Lunak</t>
   </si>
   <si>
-    <t>SMK Negeri 1 Contoh</t>
-  </si>
-  <si>
-    <t>Belum Lulus</t>
-  </si>
-  <si>
-    <t>2024</t>
-  </si>
-  <si>
-    <t>081111111111</t>
-  </si>
-  <si>
-    <t>Jl. Melati No. 1, Jakarta</t>
-  </si>
-  <si>
-    <t>Rudi Hermawan</t>
-  </si>
-  <si>
-    <t>2000000002</t>
-  </si>
-  <si>
-    <t>Teknik Komputer dan Jaringan</t>
-  </si>
-  <si>
-    <t>081222222222</t>
-  </si>
-  <si>
-    <t>Jl. Mawar No. 2, Bandung</t>
-  </si>
-  <si>
-    <t>Ani Susanti</t>
-  </si>
-  <si>
-    <t>2000000003</t>
+    <t>Lulus</t>
+  </si>
+  <si>
+    <t>Jl. Contoh No. 2, Bandung</t>
+  </si>
+  <si>
+    <t>Ayu Lestari</t>
   </si>
   <si>
     <t>Akuntansi</t>
-  </si>
-  <si>
-    <t>Lulus</t>
-  </si>
-  <si>
-    <t>2023</t>
-  </si>
-  <si>
-    <t>081333333333</t>
-  </si>
-  <si>
-    <t>Jl. Dahlia No. 3, Surabaya</t>
-  </si>
-  <si>
-    <t>Fajar Nugroho</t>
-  </si>
-  <si>
-    <t>2000000004</t>
-  </si>
-  <si>
-    <t>Multimedia</t>
-  </si>
-  <si>
-    <t>Rina Maharani</t>
-  </si>
-  <si>
-    <t>2000000005</t>
-  </si>
-  <si>
-    <t>Bisnis Digital</t>
   </si>
 </sst>
 </file>
@@ -456,10 +402,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -478,130 +424,64 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="B2">
+        <v>5001234567</v>
+      </c>
+      <c r="C2" t="s">
         <v>7</v>
       </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2">
+        <v>2025</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:8">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B3">
+        <v>5001234568</v>
+      </c>
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
+      <c r="E3">
+        <v>2024</v>
       </c>
       <c r="F3" t="s">
         <v>13</v>
       </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
-      </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
+        <v>14</v>
+      </c>
+      <c r="B4">
+        <v>5001234569</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F6" t="s">
-        <v>25</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>2025</v>
+      </c>
+      <c r="F4"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>